<commit_message>
Added some minor color functions to toolbox, updated descriptions of land use categories, added new transformers for pastures, fixed some bugs in BCL, and fixed a bug in sampling unit around trajgroups
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D111AA-CE75-364C-8638-1EC89673CD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF57E8B-F4A7-C54A-900E-AC92E68F14CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3280" yWindow="760" windowWidth="34200" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="11300" yWindow="500" windowWidth="34460" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7011,18 +7011,18 @@
     <col min="8" max="8" width="15.1640625" style="4" customWidth="1"/>
     <col min="9" max="9" width="11.5" style="5" customWidth="1"/>
     <col min="10" max="11" width="13.33203125" style="4" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" style="5" hidden="1" customWidth="1"/>
-    <col min="13" max="14" width="13.33203125" style="4" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="21.1640625" style="5" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="21.1640625" style="4" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="4" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" style="5" hidden="1" customWidth="1"/>
-    <col min="19" max="20" width="13.33203125" style="4" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="9.1640625" style="5" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="13.33203125" style="4" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="9.1640625" style="5" hidden="1" customWidth="1"/>
-    <col min="25" max="26" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" style="5" customWidth="1"/>
+    <col min="13" max="14" width="13.33203125" style="4" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" style="5" customWidth="1"/>
+    <col min="16" max="16" width="21.1640625" style="4" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" style="5" customWidth="1"/>
+    <col min="19" max="20" width="13.33203125" style="4" customWidth="1"/>
+    <col min="21" max="21" width="9.1640625" style="5" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" style="4" customWidth="1"/>
+    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" style="5" customWidth="1"/>
+    <col min="25" max="26" width="13.33203125" style="4" customWidth="1"/>
     <col min="27" max="27" width="24" style="24" customWidth="1"/>
     <col min="28" max="28" width="64.5" style="47" customWidth="1"/>
     <col min="29" max="29" width="14.6640625" style="48" customWidth="1"/>

</xml_diff>

<commit_message>
intermediate updates to IPCC CRT map
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D71ADE8-473B-F742-851A-8F31AB2988B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3EAD991-B009-C741-B026-89AF73E74A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="760" windowWidth="34480" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="1240" yWindow="760" windowWidth="34480" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed a minor bug in BCL demand adjustment, updated Carbon Ledger workbook variables, and fixed some bugs in strategies
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3EAD991-B009-C741-B026-89AF73E74A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23EC696A-A193-624B-9453-D312CE5757B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="760" windowWidth="34480" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="-960" yWindow="760" windowWidth="34480" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="520">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -922,9 +922,6 @@
     <t>Area of remaining (from simulation initialization) forest that is protected.</t>
   </si>
   <si>
-    <t>Total biomass (mass units) removals needed to satisfy fuelwood and harvested wood products demands.</t>
-  </si>
-  <si>
     <t>Latex Variable</t>
   </si>
   <si>
@@ -1030,9 +1027,6 @@
     <t>G(t, v)</t>
   </si>
   <si>
-    <t>s_{rmv}(t)</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -1570,9 +1564,6 @@
     <t>vec_total_removals_demanded_adjusted</t>
   </si>
   <si>
-    <t>Unmet demand from removals could lead to reductions in demand going forward as consumers switch to different fuels. The behavioral adjustment factor allows this behavior to be reflected in changes to demands. A value of $\beta = 1$ means that shifts incurred in the previous time period are totally adopted, while a value of $\beta = 0$ means that exogenous demands remain.</t>
-  </si>
-  <si>
     <t>z:\beta</t>
   </si>
   <si>
@@ -1595,6 +1586,21 @@
   </si>
   <si>
     <t>\psi_d(t)</t>
+  </si>
+  <si>
+    <t>\hat{d}(t)</t>
+  </si>
+  <si>
+    <t>Total exogenously specified biomass (mass units) removals needed to satisfy fuelwood and harvested wood products demands.</t>
+  </si>
+  <si>
+    <t>Total biomass (mass units) removals needed to satisfy fuelwood and harvested wood products demands, adjusted endogenously based on behavior changes.</t>
+  </si>
+  <si>
+    <t>s(t)</t>
+  </si>
+  <si>
+    <t>Vector ($n_T$)  storing removal behavioral adjustment factor (RBAF). Unmet demand from removals could lead to reductions in demand going forward as consumers switch to different fuels. The behavioral adjustment factor allows this behavior to be reflected in changes to demands. A value of $\beta = 1$ means that shifts incurred in the previous time period are totally adopted, while a value of $\beta = 0$ means that exogenous demands remain.</t>
   </si>
 </sst>
 </file>
@@ -1901,11 +1907,17 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1913,14 +1925,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2494,12 +2500,12 @@
         <v>29</v>
       </c>
       <c r="M1" s="61"/>
-      <c r="N1" s="55" t="s">
+      <c r="N1" s="57" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
       <c r="R1" s="61" t="s">
         <v>48</v>
       </c>
@@ -7059,16 +7065,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AC1:AH1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="R1:T1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="N1:Q1"/>
-    <mergeCell ref="AC1:AH1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="R1:T1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7092,16 +7098,16 @@
     <col min="11" max="11" width="14" style="4" customWidth="1"/>
     <col min="12" max="12" width="11.83203125" style="5" customWidth="1"/>
     <col min="13" max="14" width="13.33203125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="21.1640625" style="5" customWidth="1"/>
-    <col min="16" max="16" width="21.1640625" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" style="5" customWidth="1"/>
-    <col min="19" max="20" width="13.33203125" style="4" customWidth="1"/>
-    <col min="21" max="21" width="9.1640625" style="5" customWidth="1"/>
-    <col min="22" max="22" width="13.33203125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
-    <col min="24" max="24" width="9.1640625" style="5" customWidth="1"/>
-    <col min="25" max="26" width="13.33203125" style="4" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="21.1640625" style="4" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="19" max="20" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="12.5" style="4" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="25" max="26" width="13.33203125" style="4" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="26.5" style="24" customWidth="1"/>
     <col min="28" max="28" width="64.5" style="47" customWidth="1"/>
     <col min="29" max="29" width="14.6640625" style="48" customWidth="1"/>
@@ -7161,10 +7167,10 @@
       <c r="H2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="55">
+      <c r="I2" s="57">
         <v>150</v>
       </c>
-      <c r="J2" s="55"/>
+      <c r="J2" s="57"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
@@ -7198,10 +7204,10 @@
       <c r="H3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="55">
+      <c r="I3" s="57">
         <v>30</v>
       </c>
-      <c r="J3" s="55"/>
+      <c r="J3" s="57"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
@@ -7259,11 +7265,11 @@
       <c r="Z4" s="20"/>
       <c r="AB4" s="40"/>
       <c r="AC4" s="27"/>
-      <c r="AE4" s="54" t="s">
+      <c r="AE4" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="AF4" s="54"/>
-      <c r="AG4" s="54"/>
+      <c r="AF4" s="56"/>
+      <c r="AG4" s="56"/>
       <c r="AL4" t="s">
         <v>94</v>
       </c>
@@ -7279,7 +7285,7 @@
     </row>
     <row r="5" spans="1:41" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="50" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>155</v>
@@ -7293,43 +7299,43 @@
       <c r="F5" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="G5" s="53" t="s">
+      <c r="G5" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="53"/>
+      <c r="H5" s="58"/>
       <c r="I5" s="17"/>
-      <c r="J5" s="53" t="s">
+      <c r="J5" s="58" t="s">
         <v>64</v>
       </c>
-      <c r="K5" s="53"/>
-      <c r="M5" s="53" t="s">
+      <c r="K5" s="58"/>
+      <c r="M5" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="53"/>
-      <c r="P5" s="53" t="s">
+      <c r="N5" s="58"/>
+      <c r="P5" s="58" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" s="53"/>
-      <c r="S5" s="53" t="s">
+      <c r="Q5" s="58"/>
+      <c r="S5" s="58" t="s">
         <v>83</v>
       </c>
-      <c r="T5" s="53"/>
-      <c r="V5" s="53" t="s">
+      <c r="T5" s="58"/>
+      <c r="V5" s="58" t="s">
         <v>84</v>
       </c>
-      <c r="W5" s="53"/>
-      <c r="Y5" s="53" t="s">
+      <c r="W5" s="58"/>
+      <c r="Y5" s="58" t="s">
         <v>135</v>
       </c>
-      <c r="Z5" s="53"/>
+      <c r="Z5" s="58"/>
       <c r="AA5" s="24" t="s">
+        <v>293</v>
+      </c>
+      <c r="AB5" s="40" t="s">
         <v>294</v>
       </c>
-      <c r="AB5" s="40" t="s">
-        <v>295</v>
-      </c>
       <c r="AC5" s="27" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AD5" s="36" t="s">
         <v>227</v>
@@ -7427,7 +7433,7 @@
     </row>
     <row r="7" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B7" s="38" t="s">
         <v>156</v>
@@ -7493,13 +7499,13 @@
         <v>249360</v>
       </c>
       <c r="AA7" s="38" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AB7" s="42" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AC7" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE7" s="19">
         <v>0.01</v>
@@ -7526,7 +7532,7 @@
     </row>
     <row r="8" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B8" s="38" t="s">
         <v>157</v>
@@ -7594,13 +7600,13 @@
         <v>249801</v>
       </c>
       <c r="AA8" s="38" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="AB8" s="42" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AC8" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE8" s="19">
         <v>0.05</v>
@@ -7627,7 +7633,7 @@
     </row>
     <row r="9" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>220</v>
@@ -7681,13 +7687,13 @@
         <v>116</v>
       </c>
       <c r="AA9" s="38" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="AB9" s="42" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AC9" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE9" s="19">
         <v>0.12</v>
@@ -7714,7 +7720,7 @@
     </row>
     <row r="10" spans="1:41" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B10" s="38" t="s">
         <v>219</v>
@@ -7760,7 +7766,7 @@
         <v>286</v>
       </c>
       <c r="AC10" s="43" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AE10" s="19">
         <v>0.2</v>
@@ -7775,7 +7781,7 @@
     </row>
     <row r="11" spans="1:41" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B11" s="38" t="s">
         <v>217</v>
@@ -7821,7 +7827,7 @@
         <v>287</v>
       </c>
       <c r="AC11" s="43" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AE11" s="19">
         <v>0.2</v>
@@ -7836,10 +7842,10 @@
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A12" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C12" s="28"/>
       <c r="G12" s="4">
@@ -7899,10 +7905,10 @@
         <v>116</v>
       </c>
       <c r="AA12" s="38" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="AB12" s="42" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="AC12" s="43"/>
       <c r="AE12" s="19"/>
@@ -7911,7 +7917,7 @@
     </row>
     <row r="13" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>218</v>
@@ -7950,7 +7956,7 @@
         <v>288</v>
       </c>
       <c r="AC13" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE13" s="19">
         <v>0.36</v>
@@ -7965,7 +7971,7 @@
     </row>
     <row r="14" spans="1:41" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B14" s="38" t="s">
         <v>158</v>
@@ -8034,10 +8040,10 @@
       </c>
       <c r="AA14" s="38"/>
       <c r="AB14" s="51" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="AC14" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE14" s="19"/>
       <c r="AF14" s="19"/>
@@ -8045,7 +8051,7 @@
     </row>
     <row r="15" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B15" s="38" t="s">
         <v>221</v>
@@ -8078,13 +8084,13 @@
         <v>0.7</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AB15" s="42" t="s">
         <v>289</v>
       </c>
       <c r="AC15" s="43" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="AE15" s="19">
         <v>0.6</v>
@@ -8099,7 +8105,7 @@
     </row>
     <row r="16" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B16" s="38" t="s">
         <v>241</v>
@@ -8156,13 +8162,13 @@
         <v>9</v>
       </c>
       <c r="AA16" s="38" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="AB16" s="42" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AC16" s="43" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AE16" s="19"/>
       <c r="AF16" s="19"/>
@@ -8170,7 +8176,7 @@
     </row>
     <row r="17" spans="1:33" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B17" s="38" t="s">
         <v>277</v>
@@ -8235,13 +8241,13 @@
         <v>1.728</v>
       </c>
       <c r="AA17" s="38" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="AB17" s="42" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AC17" s="43" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AE17" s="19"/>
       <c r="AF17" s="19"/>
@@ -8249,10 +8255,10 @@
     </row>
     <row r="18" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C18" s="31" t="s">
         <v>162</v>
@@ -8267,13 +8273,13 @@
         <v>0.37800893000000002</v>
       </c>
       <c r="AA18" s="38" t="s">
+        <v>400</v>
+      </c>
+      <c r="AB18" s="42" t="s">
         <v>402</v>
       </c>
-      <c r="AB18" s="42" t="s">
-        <v>404</v>
-      </c>
       <c r="AC18" s="43" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="AE18" s="19">
         <v>1.8</v>
@@ -8288,15 +8294,15 @@
     </row>
     <row r="19" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B19" s="38" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C19" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="52" t="s">
+      <c r="E19" s="55" t="s">
         <v>118</v>
       </c>
       <c r="F19" s="10" t="s">
@@ -8309,13 +8315,13 @@
         <v>0.47800893</v>
       </c>
       <c r="AA19" s="38" t="s">
+        <v>401</v>
+      </c>
+      <c r="AB19" s="42" t="s">
         <v>403</v>
       </c>
-      <c r="AB19" s="42" t="s">
-        <v>405</v>
-      </c>
       <c r="AC19" s="43" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="AE19" s="19">
         <v>3</v>
@@ -8330,7 +8336,7 @@
     </row>
     <row r="20" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B20" s="38" t="s">
         <v>222</v>
@@ -8338,7 +8344,7 @@
       <c r="C20" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E20" s="52"/>
+      <c r="E20" s="55"/>
       <c r="F20" s="10" t="s">
         <v>138</v>
       </c>
@@ -8352,7 +8358,7 @@
         <v>285</v>
       </c>
       <c r="AC20" s="43" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="AE20" s="19">
         <v>6</v>
@@ -8367,7 +8373,7 @@
     </row>
     <row r="21" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>224</v>
@@ -8385,13 +8391,13 @@
         <v>100</v>
       </c>
       <c r="AA21" s="38" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="AB21" s="42" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="AC21" s="43" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AE21" s="19">
         <v>10</v>
@@ -8406,7 +8412,7 @@
     </row>
     <row r="22" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B22" s="38" t="s">
         <v>226</v>
@@ -8424,13 +8430,13 @@
         <v>0.25</v>
       </c>
       <c r="AA22" s="38" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="AB22" s="42" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="AC22" s="44" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="AE22" s="19"/>
       <c r="AF22" s="19"/>
@@ -8438,7 +8444,7 @@
     </row>
     <row r="23" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B23" s="38" t="s">
         <v>269</v>
@@ -8458,13 +8464,13 @@
         <v>37.800893000000002</v>
       </c>
       <c r="AA23" s="38" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="AB23" s="42" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="AC23" s="43" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="AE23" s="19">
         <v>12</v>
@@ -8479,7 +8485,7 @@
     </row>
     <row r="24" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B24" s="38" t="s">
         <v>225</v>
@@ -8499,13 +8505,13 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA24" s="38" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="AB24" s="42" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="AC24" s="43" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AE24" s="19">
         <v>13.5</v>
@@ -8534,7 +8540,7 @@
     </row>
     <row r="26" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B26" s="38" t="s">
         <v>159</v>
@@ -8588,13 +8594,13 @@
         <v>49500</v>
       </c>
       <c r="AA26" s="38" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="AB26" s="42" t="s">
         <v>290</v>
       </c>
       <c r="AC26" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE26" s="19">
         <v>10</v>
@@ -8609,7 +8615,7 @@
     </row>
     <row r="27" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>268</v>
@@ -8649,13 +8655,13 @@
         <v>0</v>
       </c>
       <c r="AA27" s="38" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="AB27" s="42" t="s">
         <v>291</v>
       </c>
       <c r="AC27" s="43" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AE27" s="19">
         <v>6</v>
@@ -8670,7 +8676,7 @@
     </row>
     <row r="28" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B28" s="38" t="s">
         <v>160</v>
@@ -8738,13 +8744,13 @@
         <v>49500</v>
       </c>
       <c r="AA28" s="38" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="AB28" s="42" t="s">
         <v>292</v>
       </c>
       <c r="AC28" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AE28" s="19">
         <v>3</v>
@@ -8790,7 +8796,7 @@
     </row>
     <row r="30" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B30" s="38" t="s">
         <v>267</v>
@@ -8798,7 +8804,7 @@
       <c r="C30" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E30" s="52" t="s">
+      <c r="E30" s="55" t="s">
         <v>170</v>
       </c>
       <c r="F30" s="25" t="s">
@@ -8811,26 +8817,26 @@
         <v>0.92</v>
       </c>
       <c r="AA30" s="38" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB30" s="42" t="s">
         <v>311</v>
       </c>
-      <c r="AB30" s="42" t="s">
-        <v>312</v>
-      </c>
       <c r="AC30" s="43" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="31" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B31" s="38" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C31" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E31" s="52"/>
+      <c r="E31" s="55"/>
       <c r="F31" s="25" t="s">
         <v>171</v>
       </c>
@@ -8847,21 +8853,21 @@
         <v>2E-3</v>
       </c>
       <c r="AA31" s="38" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="AB31" s="42" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="AC31" s="43" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="32" spans="1:33" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B32" s="38" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C32" s="31" t="s">
         <v>162</v>
@@ -8872,37 +8878,37 @@
         <v>0.61538461538461542</v>
       </c>
       <c r="AA32" s="38" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="AB32" s="42" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="AC32" s="43" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="33" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B33" s="38" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E33" s="26"/>
       <c r="G33" s="4">
         <v>0.5</v>
       </c>
       <c r="AA33" s="38" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="AB33" s="42" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="AC33" s="43" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="34" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -8928,7 +8934,7 @@
     </row>
     <row r="35" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B35" s="38" t="s">
         <v>168</v>
@@ -8964,21 +8970,21 @@
         <v>279</v>
       </c>
       <c r="AB35" s="42" t="s">
-        <v>293</v>
+        <v>516</v>
       </c>
       <c r="AC35" s="43" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="36" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B36" s="38" t="s">
-        <v>508</v>
-      </c>
-      <c r="C36" s="28" t="s">
-        <v>174</v>
+        <v>506</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>163</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>53</v>
@@ -9011,24 +9017,24 @@
         <v>224809.55611554152</v>
       </c>
       <c r="AA36" s="38" t="s">
-        <v>279</v>
+        <v>515</v>
       </c>
       <c r="AB36" s="42" t="s">
-        <v>293</v>
+        <v>517</v>
       </c>
       <c r="AC36" s="43" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B37" s="38" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="G37" s="4">
         <v>0.14000000000000001</v>
@@ -9052,24 +9058,24 @@
         <v>0.14199999999999999</v>
       </c>
       <c r="AA37" s="38" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="AB37" s="42" t="s">
+        <v>510</v>
+      </c>
+      <c r="AC37" s="43" t="s">
         <v>513</v>
-      </c>
-      <c r="AC37" s="43" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="38" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B38" s="38" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="G38" s="4">
         <v>1</v>
@@ -9093,21 +9099,21 @@
         <v>1</v>
       </c>
       <c r="AA38" s="38" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="AB38" s="42" t="s">
-        <v>509</v>
+        <v>519</v>
       </c>
       <c r="AC38" s="43" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="39" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C39" s="31" t="s">
         <v>162</v>
@@ -9135,13 +9141,13 @@
         <v>0.5</v>
       </c>
       <c r="AA39" s="38" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="AB39" s="42" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="AC39" s="43" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="40" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -9150,10 +9156,10 @@
     </row>
     <row r="41" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B41" s="38" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="C41" s="28" t="s">
         <v>174</v>
@@ -9189,13 +9195,13 @@
         <v>8.9210141315691077E-2</v>
       </c>
       <c r="AA41" s="38" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="AB41" s="42" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="AC41" s="43" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -9302,12 +9308,12 @@
     </row>
     <row r="45" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B45" s="37" t="s">
-        <v>296</v>
-      </c>
-      <c r="C45" s="56" t="s">
+        <v>295</v>
+      </c>
+      <c r="C45" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F45" s="14" t="s">
@@ -9393,23 +9399,23 @@
         <v>85</v>
       </c>
       <c r="AA45" s="38" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AB45" s="42" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="AC45" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="46" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B46" s="38" t="s">
-        <v>297</v>
-      </c>
-      <c r="C46" s="56"/>
+        <v>296</v>
+      </c>
+      <c r="C46" s="53"/>
       <c r="F46" s="14" t="s">
         <v>69</v>
       </c>
@@ -9492,23 +9498,23 @@
         <v>80</v>
       </c>
       <c r="AA46" s="38" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="AB46" s="42" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="AC46" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B47" s="38" t="s">
-        <v>298</v>
-      </c>
-      <c r="C47" s="56"/>
+        <v>297</v>
+      </c>
+      <c r="C47" s="53"/>
       <c r="F47" s="14" t="s">
         <v>79</v>
       </c>
@@ -9590,18 +9596,18 @@
         <v>92</v>
       </c>
       <c r="AA47" s="38" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AB47" s="42" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="AC47" s="43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="38"/>
-      <c r="C48" s="56"/>
+      <c r="C48" s="53"/>
       <c r="F48" s="14" t="s">
         <v>80</v>
       </c>
@@ -9694,12 +9700,12 @@
     </row>
     <row r="50" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B50" s="57" t="s">
+        <v>405</v>
+      </c>
+      <c r="B50" s="54" t="s">
         <v>189</v>
       </c>
-      <c r="C50" s="56" t="s">
+      <c r="C50" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F50" s="14" t="s">
@@ -9736,15 +9742,15 @@
         <v>280</v>
       </c>
       <c r="AB50" s="42" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="AC50" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="51" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="57"/>
-      <c r="C51" s="56"/>
+      <c r="B51" s="54"/>
+      <c r="C51" s="53"/>
       <c r="F51" s="14" t="s">
         <v>194</v>
       </c>
@@ -9780,8 +9786,8 @@
       <c r="AC51" s="43"/>
     </row>
     <row r="52" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B52" s="57"/>
-      <c r="C52" s="56"/>
+      <c r="B52" s="54"/>
+      <c r="C52" s="53"/>
       <c r="F52" s="14" t="s">
         <v>195</v>
       </c>
@@ -9817,8 +9823,8 @@
       <c r="AC52" s="43"/>
     </row>
     <row r="53" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="57"/>
-      <c r="C53" s="56"/>
+      <c r="B53" s="54"/>
+      <c r="C53" s="53"/>
       <c r="F53" s="14" t="s">
         <v>196</v>
       </c>
@@ -9855,7 +9861,7 @@
     </row>
     <row r="54" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B54" s="38" t="s">
         <v>190</v>
@@ -9896,10 +9902,10 @@
         <v>281</v>
       </c>
       <c r="AB54" s="42" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="AC54" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="55" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -9911,15 +9917,15 @@
     </row>
     <row r="56" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B56" s="57" t="s">
+        <v>405</v>
+      </c>
+      <c r="B56" s="54" t="s">
         <v>253</v>
       </c>
-      <c r="C56" s="56" t="s">
+      <c r="C56" s="53" t="s">
         <v>174</v>
       </c>
-      <c r="E56" s="52" t="s">
+      <c r="E56" s="55" t="s">
         <v>243</v>
       </c>
       <c r="F56" s="14" t="s">
@@ -9954,19 +9960,19 @@
         <v>0</v>
       </c>
       <c r="AA56" s="38" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="AB56" s="42" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="AC56" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="57" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="57"/>
-      <c r="C57" s="56"/>
-      <c r="E57" s="52"/>
+      <c r="B57" s="54"/>
+      <c r="C57" s="53"/>
+      <c r="E57" s="55"/>
       <c r="F57" s="14" t="s">
         <v>244</v>
       </c>
@@ -10003,9 +10009,9 @@
       <c r="AC57" s="43"/>
     </row>
     <row r="58" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="57"/>
-      <c r="C58" s="56"/>
-      <c r="E58" s="52"/>
+      <c r="B58" s="54"/>
+      <c r="C58" s="53"/>
+      <c r="E58" s="55"/>
       <c r="F58" s="14" t="s">
         <v>245</v>
       </c>
@@ -10042,9 +10048,9 @@
       <c r="AC58" s="43"/>
     </row>
     <row r="59" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="57"/>
-      <c r="C59" s="56"/>
-      <c r="E59" s="52"/>
+      <c r="B59" s="54"/>
+      <c r="C59" s="53"/>
+      <c r="E59" s="55"/>
       <c r="F59" s="14" t="s">
         <v>246</v>
       </c>
@@ -10082,7 +10088,7 @@
     </row>
     <row r="60" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B60" s="38" t="s">
         <v>254</v>
@@ -10120,18 +10126,18 @@
         <v>0</v>
       </c>
       <c r="AA60" s="38" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AB60" s="42" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="AC60" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="61" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B61" s="38" t="s">
         <v>256</v>
@@ -10167,13 +10173,13 @@
         <v>0</v>
       </c>
       <c r="AA61" s="38" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="AB61" s="42" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="AC61" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="62" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -10183,12 +10189,12 @@
     </row>
     <row r="63" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B63" s="57" t="s">
+        <v>405</v>
+      </c>
+      <c r="B63" s="54" t="s">
         <v>191</v>
       </c>
-      <c r="C63" s="56" t="s">
+      <c r="C63" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F63" s="14" t="s">
@@ -10226,15 +10232,15 @@
         <v>282</v>
       </c>
       <c r="AB63" s="42" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="AC63" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="64" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B64" s="57"/>
-      <c r="C64" s="56"/>
+      <c r="B64" s="54"/>
+      <c r="C64" s="53"/>
       <c r="F64" s="14" t="s">
         <v>198</v>
       </c>
@@ -10271,8 +10277,8 @@
       <c r="AC64" s="43"/>
     </row>
     <row r="65" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B65" s="57"/>
-      <c r="C65" s="56"/>
+      <c r="B65" s="54"/>
+      <c r="C65" s="53"/>
       <c r="F65" s="14" t="s">
         <v>199</v>
       </c>
@@ -10309,8 +10315,8 @@
       <c r="AC65" s="43"/>
     </row>
     <row r="66" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B66" s="57"/>
-      <c r="C66" s="56"/>
+      <c r="B66" s="54"/>
+      <c r="C66" s="53"/>
       <c r="F66" s="14" t="s">
         <v>200</v>
       </c>
@@ -10348,7 +10354,7 @@
     </row>
     <row r="67" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B67" s="38" t="s">
         <v>192</v>
@@ -10389,10 +10395,10 @@
         <v>283</v>
       </c>
       <c r="AB67" s="42" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="AC67" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="68" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -10402,12 +10408,12 @@
     </row>
     <row r="69" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B69" s="57" t="s">
+        <v>405</v>
+      </c>
+      <c r="B69" s="54" t="s">
         <v>178</v>
       </c>
-      <c r="C69" s="56" t="s">
+      <c r="C69" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F69" s="14" t="s">
@@ -10442,18 +10448,18 @@
         <v>0.6</v>
       </c>
       <c r="AA69" s="38" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="AB69" s="42" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="AC69" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="70" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B70" s="57"/>
-      <c r="C70" s="56"/>
+      <c r="B70" s="54"/>
+      <c r="C70" s="53"/>
       <c r="F70" s="14" t="s">
         <v>91</v>
       </c>
@@ -10488,8 +10494,8 @@
       <c r="AC70" s="43"/>
     </row>
     <row r="71" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="57"/>
-      <c r="C71" s="56"/>
+      <c r="B71" s="54"/>
+      <c r="C71" s="53"/>
       <c r="F71" s="14" t="s">
         <v>92</v>
       </c>
@@ -10523,8 +10529,8 @@
       <c r="AC71" s="43"/>
     </row>
     <row r="72" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B72" s="57"/>
-      <c r="C72" s="56"/>
+      <c r="B72" s="54"/>
+      <c r="C72" s="53"/>
       <c r="F72" s="14" t="s">
         <v>93</v>
       </c>
@@ -10558,10 +10564,10 @@
     </row>
     <row r="73" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B73" s="38" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C73" s="31" t="s">
         <v>162</v>
@@ -10570,13 +10576,13 @@
         <v>49</v>
       </c>
       <c r="AA73" s="38" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="AB73" s="42" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="AC73" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="74" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -10586,12 +10592,12 @@
     </row>
     <row r="75" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B75" s="57" t="s">
+        <v>405</v>
+      </c>
+      <c r="B75" s="54" t="s">
         <v>230</v>
       </c>
-      <c r="C75" s="56" t="s">
+      <c r="C75" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F75" s="14" t="s">
@@ -10629,15 +10635,15 @@
         <v>284</v>
       </c>
       <c r="AB75" s="42" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="AC75" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="76" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="57"/>
-      <c r="C76" s="56"/>
+      <c r="B76" s="54"/>
+      <c r="C76" s="53"/>
       <c r="F76" s="14" t="s">
         <v>110</v>
       </c>
@@ -10670,9 +10676,9 @@
       <c r="AC76" s="43"/>
     </row>
     <row r="77" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B77" s="57"/>
-      <c r="C77" s="56"/>
-      <c r="E77" s="52"/>
+      <c r="B77" s="54"/>
+      <c r="C77" s="53"/>
+      <c r="E77" s="55"/>
       <c r="F77" s="14" t="s">
         <v>111</v>
       </c>
@@ -10701,9 +10707,9 @@
       <c r="AC77" s="43"/>
     </row>
     <row r="78" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="57"/>
-      <c r="C78" s="56"/>
-      <c r="E78" s="52"/>
+      <c r="B78" s="54"/>
+      <c r="C78" s="53"/>
+      <c r="E78" s="55"/>
       <c r="F78" s="14" t="s">
         <v>112</v>
       </c>
@@ -10732,14 +10738,14 @@
       <c r="AC78" s="43"/>
     </row>
     <row r="79" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E79" s="52"/>
+      <c r="E79" s="55"/>
       <c r="F79" s="14"/>
       <c r="AB79" s="42"/>
       <c r="AC79" s="43"/>
     </row>
     <row r="80" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B80" s="38" t="s">
         <v>228</v>
@@ -10778,13 +10784,13 @@
         <v>0</v>
       </c>
       <c r="AA80" s="38" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="AB80" s="42" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="AC80" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="81" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -10903,7 +10909,7 @@
     </row>
     <row r="84" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B84" s="38" t="s">
         <v>229</v>
@@ -10942,13 +10948,13 @@
         <v>0</v>
       </c>
       <c r="AA84" s="45" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="AB84" s="42" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="AC84" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AF84" t="s">
         <v>106</v>
@@ -10967,12 +10973,12 @@
     </row>
     <row r="86" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B86" s="37" t="s">
-        <v>420</v>
-      </c>
-      <c r="C86" s="56" t="s">
+        <v>418</v>
+      </c>
+      <c r="C86" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F86" s="14" t="s">
@@ -11000,13 +11006,13 @@
         <v>0</v>
       </c>
       <c r="AA86" s="38" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="AB86" s="42" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="AC86" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AD86" t="s">
         <v>86</v>
@@ -11014,12 +11020,12 @@
     </row>
     <row r="87" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B87" s="37" t="s">
-        <v>419</v>
-      </c>
-      <c r="C87" s="56"/>
+        <v>417</v>
+      </c>
+      <c r="C87" s="53"/>
       <c r="F87" s="14" t="s">
         <v>148</v>
       </c>
@@ -11080,18 +11086,18 @@
         <v>0</v>
       </c>
       <c r="AA87" s="38" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="AB87" s="42" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="AC87" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="88" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B88" s="41"/>
-      <c r="C88" s="56"/>
+      <c r="C88" s="53"/>
       <c r="E88" s="22">
         <v>0</v>
       </c>
@@ -11160,7 +11166,7 @@
     </row>
     <row r="89" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B89" s="41"/>
-      <c r="C89" s="56"/>
+      <c r="C89" s="53"/>
       <c r="E89" s="22">
         <v>1</v>
       </c>
@@ -11229,7 +11235,7 @@
     </row>
     <row r="90" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B90" s="41"/>
-      <c r="C90" s="56"/>
+      <c r="C90" s="53"/>
       <c r="E90" s="22">
         <v>2</v>
       </c>
@@ -11321,12 +11327,12 @@
     </row>
     <row r="92" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B92" s="37" t="s">
-        <v>418</v>
-      </c>
-      <c r="C92" s="56" t="s">
+        <v>416</v>
+      </c>
+      <c r="C92" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F92" s="14" t="s">
@@ -11385,23 +11391,23 @@
         <v>0.6</v>
       </c>
       <c r="AA92" s="37" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="AB92" s="42" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="AC92" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="93" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B93" s="37" t="s">
-        <v>417</v>
-      </c>
-      <c r="C93" s="56"/>
+        <v>415</v>
+      </c>
+      <c r="C93" s="53"/>
       <c r="F93" s="14" t="s">
         <v>132</v>
       </c>
@@ -11458,18 +11464,18 @@
         <v>0.36</v>
       </c>
       <c r="AA93" s="37" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AB93" s="42" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="AC93" s="43" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="94" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B94" s="37"/>
-      <c r="C94" s="56"/>
+      <c r="C94" s="53"/>
       <c r="F94" s="14" t="s">
         <v>133</v>
       </c>
@@ -11531,7 +11537,7 @@
     </row>
     <row r="95" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B95" s="41"/>
-      <c r="C95" s="56"/>
+      <c r="C95" s="53"/>
       <c r="F95" s="14" t="s">
         <v>134</v>
       </c>
@@ -11598,12 +11604,12 @@
     </row>
     <row r="97" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B97" s="58" t="s">
-        <v>482</v>
-      </c>
-      <c r="C97" s="56" t="s">
+        <v>405</v>
+      </c>
+      <c r="B97" s="52" t="s">
+        <v>480</v>
+      </c>
+      <c r="C97" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F97" s="14" t="s">
@@ -11638,18 +11644,18 @@
         <v>9.8621113109027395E-2</v>
       </c>
       <c r="AA97" s="37" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="AB97" s="42" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="AC97" s="43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="98" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B98" s="58"/>
-      <c r="C98" s="56"/>
+      <c r="B98" s="52"/>
+      <c r="C98" s="53"/>
       <c r="F98" s="14" t="s">
         <v>203</v>
       </c>
@@ -11686,8 +11692,8 @@
       <c r="AC98" s="43"/>
     </row>
     <row r="99" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="58"/>
-      <c r="C99" s="56"/>
+      <c r="B99" s="52"/>
+      <c r="C99" s="53"/>
       <c r="F99" s="14" t="s">
         <v>204</v>
       </c>
@@ -11724,8 +11730,8 @@
       <c r="AC99" s="43"/>
     </row>
     <row r="100" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="58"/>
-      <c r="C100" s="56"/>
+      <c r="B100" s="52"/>
+      <c r="C100" s="53"/>
       <c r="F100" s="14" t="s">
         <v>205</v>
       </c>
@@ -11763,10 +11769,10 @@
     </row>
     <row r="101" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B101" s="37" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C101" s="28"/>
       <c r="F101" s="14"/>
@@ -11799,13 +11805,13 @@
         <v>0.17633270956878355</v>
       </c>
       <c r="AA101" s="37" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="AB101" s="42" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="AC101" s="43" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="102" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -11815,12 +11821,12 @@
     </row>
     <row r="103" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B103" s="58" t="s">
+        <v>405</v>
+      </c>
+      <c r="B103" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="C103" s="56" t="s">
+      <c r="C103" s="53" t="s">
         <v>174</v>
       </c>
       <c r="F103" s="14" t="s">
@@ -11855,18 +11861,18 @@
         <v>113.71737449773644</v>
       </c>
       <c r="AA103" s="38" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AB103" s="42" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="AC103" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="104" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B104" s="58"/>
-      <c r="C104" s="56"/>
+      <c r="B104" s="52"/>
+      <c r="C104" s="53"/>
       <c r="F104" s="14" t="s">
         <v>71</v>
       </c>
@@ -11903,8 +11909,8 @@
       <c r="AC104" s="43"/>
     </row>
     <row r="105" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B105" s="58"/>
-      <c r="C105" s="56"/>
+      <c r="B105" s="52"/>
+      <c r="C105" s="53"/>
       <c r="F105" s="14" t="s">
         <v>72</v>
       </c>
@@ -11941,8 +11947,8 @@
       <c r="AC105" s="43"/>
     </row>
     <row r="106" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B106" s="58"/>
-      <c r="C106" s="56"/>
+      <c r="B106" s="52"/>
+      <c r="C106" s="53"/>
       <c r="F106" s="14" t="s">
         <v>81</v>
       </c>
@@ -11986,12 +11992,12 @@
     </row>
     <row r="108" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B108" s="58" t="s">
+        <v>405</v>
+      </c>
+      <c r="B108" s="52" t="s">
         <v>207</v>
       </c>
-      <c r="C108" s="56" t="s">
+      <c r="C108" s="53" t="s">
         <v>174</v>
       </c>
       <c r="E108" s="26"/>
@@ -12027,18 +12033,18 @@
         <v>28.429343624434111</v>
       </c>
       <c r="AA108" s="38" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="AB108" s="42" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="AC108" s="43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="109" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B109" s="58"/>
-      <c r="C109" s="56"/>
+      <c r="B109" s="52"/>
+      <c r="C109" s="53"/>
       <c r="E109" s="26"/>
       <c r="F109" s="14" t="s">
         <v>209</v>
@@ -12076,8 +12082,8 @@
       <c r="AC109" s="43"/>
     </row>
     <row r="110" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B110" s="58"/>
-      <c r="C110" s="56"/>
+      <c r="B110" s="52"/>
+      <c r="C110" s="53"/>
       <c r="E110" s="26"/>
       <c r="F110" s="14" t="s">
         <v>210</v>
@@ -12115,8 +12121,8 @@
       <c r="AC110" s="43"/>
     </row>
     <row r="111" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B111" s="58"/>
-      <c r="C111" s="56"/>
+      <c r="B111" s="52"/>
+      <c r="C111" s="53"/>
       <c r="E111" s="26"/>
       <c r="F111" s="14" t="s">
         <v>211</v>
@@ -12256,7 +12262,7 @@
     </row>
     <row r="116" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B116" s="38" t="s">
         <v>232</v>
@@ -12324,18 +12330,18 @@
         <v>24936000</v>
       </c>
       <c r="AA116" s="38" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="AB116" s="42" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AC116" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="117" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B117" s="38" t="s">
         <v>181</v>
@@ -12401,18 +12407,18 @@
         <v>0.8507753625870188</v>
       </c>
       <c r="AA117" s="38" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="AB117" s="42" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="AC117" s="43" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="118" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B118" s="38" t="s">
         <v>182</v>
@@ -12480,18 +12486,18 @@
         <v>0.78271333358005735</v>
       </c>
       <c r="AA118" s="38" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="AB118" s="42" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="AC118" s="43" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="119" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B119" s="38" t="s">
         <v>233</v>
@@ -12559,18 +12565,18 @@
         <v>15569496.768312966</v>
       </c>
       <c r="AA119" s="38" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="AB119" s="42" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="AC119" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="120" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B120" s="38" t="s">
         <v>236</v>
@@ -12638,18 +12644,18 @@
         <v>62.4378279127084</v>
       </c>
       <c r="AA120" s="38" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="AB120" s="42" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="AC120" s="43" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="121" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B121" s="38" t="s">
         <v>271</v>
@@ -12717,13 +12723,13 @@
         <v>24.636934912708398</v>
       </c>
       <c r="AA121" s="38" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="AB121" s="46" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AC121" s="43" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="122" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -12754,7 +12760,7 @@
     </row>
     <row r="124" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B124" s="38" t="s">
         <v>238</v>
@@ -12827,7 +12833,7 @@
     </row>
     <row r="125" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B125" s="38" t="s">
         <v>237</v>
@@ -12867,18 +12873,18 @@
         <v>215.49749504124878</v>
       </c>
       <c r="AA125" s="38" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AB125" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="AC125" s="43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="126" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B126" s="38" t="s">
         <v>234</v>
@@ -12946,18 +12952,18 @@
         <v>15569712.265808009</v>
       </c>
       <c r="AA126" s="38" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="AB126" s="42" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="AC126" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="127" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B127" s="38" t="s">
         <v>235</v>
@@ -13025,18 +13031,18 @@
         <v>3892428.0664520022</v>
       </c>
       <c r="AA127" s="38" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="AB127" s="42" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="AC127" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="128" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B128" s="38" t="s">
         <v>270</v>
@@ -13104,18 +13110,18 @@
         <v>7242.7880378741747</v>
       </c>
       <c r="AA128" s="38" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="AB128" s="42" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="AC128" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="129" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B129" s="38" t="s">
         <v>255</v>
@@ -13183,18 +13189,18 @@
         <v>1044</v>
       </c>
       <c r="AA129" s="38" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="AB129" s="42" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="AC129" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="130" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B130" s="38" t="s">
         <v>272</v>
@@ -13262,21 +13268,21 @@
         <v>4339.1516265119217</v>
       </c>
       <c r="AA130" s="38" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="AB130" s="42" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="AC130" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="131" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B131" s="38" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C131" s="33" t="s">
         <v>163</v>
@@ -13313,18 +13319,18 @@
         <v>9682.132802972681</v>
       </c>
       <c r="AA131" s="38" t="s">
+        <v>316</v>
+      </c>
+      <c r="AB131" s="42" t="s">
         <v>317</v>
       </c>
-      <c r="AB131" s="42" t="s">
-        <v>318</v>
-      </c>
       <c r="AC131" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="132" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B132" s="38" t="s">
         <v>250</v>
@@ -13392,18 +13398,18 @@
         <v>0.4481607219000015</v>
       </c>
       <c r="AA132" s="38" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="AB132" s="42" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="AC132" s="43" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="133" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B133" s="38" t="s">
         <v>183</v>
@@ -13471,13 +13477,13 @@
         <v>4921079.9272040259</v>
       </c>
       <c r="AA133" s="38" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="AB133" s="42" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="AC133" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="134" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -13507,10 +13513,10 @@
     </row>
     <row r="136" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B136" s="38" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="C136" s="28" t="s">
         <v>174</v>
@@ -13545,21 +13551,21 @@
         <v>215127.42331256883</v>
       </c>
       <c r="AA136" s="38" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="AB136" s="42" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="AC136" s="43" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="137" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B137" s="38" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C137" s="28" t="s">
         <v>174</v>
@@ -13594,21 +13600,21 @@
         <v>9423.9320294407444</v>
       </c>
       <c r="AA137" s="38" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AB137" s="42" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="AC137" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="138" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B138" s="38" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C138" s="28" t="s">
         <v>174</v>
@@ -13645,21 +13651,21 @@
         <v>205703.4912831281</v>
       </c>
       <c r="AA138" s="38" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AB138" s="42" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="AC138" s="43" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="139" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B139" s="38" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C139" s="28" t="s">
         <v>174</v>
@@ -13694,18 +13700,18 @@
         <v>0</v>
       </c>
       <c r="AA139" s="38" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="AB139" s="42" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="AC139" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="140" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B140" s="38" t="s">
         <v>251</v>
@@ -13745,18 +13751,18 @@
         <v>192920.79914218979</v>
       </c>
       <c r="AA140" s="38" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="AB140" s="42" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="AC140" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="141" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B141" s="38" t="s">
         <v>262</v>
@@ -13796,21 +13802,21 @@
         <v>12782.692140938307</v>
       </c>
       <c r="AA141" s="38" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AB141" s="42" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="AC141" s="43" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="142" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B142" s="38" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C142" s="28" t="s">
         <v>174</v>
@@ -13847,18 +13853,18 @@
         <v>0</v>
       </c>
       <c r="AA142" s="38" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="AB142" s="42" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AC142" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="143" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B143" s="38" t="s">
         <v>258</v>
@@ -13926,18 +13932,18 @@
         <v>186224.98890231474</v>
       </c>
       <c r="AA143" s="38" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="AB143" s="42" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="AC143" s="43" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="144" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B144" s="38" t="s">
         <v>263</v>
@@ -14005,13 +14011,13 @@
         <v>186224.98890231474</v>
       </c>
       <c r="AA144" s="38" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="AB144" s="42" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="AC144" s="43" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="145" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14037,7 +14043,7 @@
     </row>
     <row r="146" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B146" s="38" t="s">
         <v>265</v>
@@ -14105,13 +14111,13 @@
         <v>0.39609788791193412</v>
       </c>
       <c r="AA146" s="38" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="AB146" s="42" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="AC146" s="43" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="AD146">
         <v>20</v>
@@ -14119,7 +14125,7 @@
     </row>
     <row r="147" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B147" s="38" t="s">
         <v>184</v>
@@ -14187,13 +14193,13 @@
         <v>3.7842301213774604E-2</v>
       </c>
       <c r="AA147" s="39" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="AB147" s="42" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="AC147" s="43" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="AD147">
         <v>20</v>
@@ -14210,7 +14216,7 @@
     </row>
     <row r="149" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B149" s="38" t="s">
         <v>186</v>
@@ -14278,13 +14284,13 @@
         <v>186224.98890231474</v>
       </c>
       <c r="AA149" s="38" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="AB149" s="42" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="AC149" s="43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="AD149">
         <v>20</v>
@@ -14292,7 +14298,7 @@
     </row>
     <row r="150" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B150" s="38" t="s">
         <v>187</v>
@@ -14360,18 +14366,18 @@
         <v>192920.79914218979</v>
       </c>
       <c r="AA150" s="38" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="AB150" s="42" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AC150" s="43" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="151" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B151" s="38" t="s">
         <v>188</v>
@@ -14439,13 +14445,13 @@
         <v>0.96529243985279167</v>
       </c>
       <c r="AA151" s="38" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AB151" s="42" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="AC151" s="43" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="152" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14475,10 +14481,10 @@
     </row>
     <row r="154" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B154" s="38" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C154" s="33" t="s">
         <v>163</v>
@@ -14543,21 +14549,21 @@
         <v>24140.541849164827</v>
       </c>
       <c r="AA154" s="38" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="AB154" s="42" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC154" s="43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="155" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B155" s="38" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C155" s="33" t="s">
         <v>163</v>
@@ -14619,18 +14625,18 @@
         <v>6035.1354622912067</v>
       </c>
       <c r="AA155" s="38" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="AB155" s="42" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="AC155" s="43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="156" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B156" s="38" t="s">
         <v>264</v>
@@ -14698,18 +14704,18 @@
         <v>46556.247225578685</v>
       </c>
       <c r="AA156" s="38" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AB156" s="42" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="AC156" s="43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="157" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B157" s="38" t="s">
         <v>176</v>
@@ -14777,18 +14783,18 @@
         <v>1859.6364113622531</v>
       </c>
       <c r="AA157" s="38" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="AB157" s="42" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="AC157" s="43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="158" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B158" s="38" t="s">
         <v>177</v>
@@ -14856,18 +14862,18 @@
         <v>1349.2490094685436</v>
       </c>
       <c r="AA158" s="38" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="AB158" s="42" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="AC158" s="43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="159" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B159" s="38" t="s">
         <v>278</v>
@@ -14932,13 +14938,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA159" s="38" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="AB159" s="42" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="AC159" s="43" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="160" spans="1:30" x14ac:dyDescent="0.2">
@@ -15018,7 +15024,7 @@
     </row>
     <row r="164" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A164" s="50" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B164" s="38" t="s">
         <v>266</v>
@@ -15055,13 +15061,13 @@
         <v>212026.86397460321</v>
       </c>
       <c r="AA164" s="38" t="s">
-        <v>329</v>
+        <v>518</v>
       </c>
       <c r="AB164" s="42" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="AC164" s="43" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="165" spans="1:30" x14ac:dyDescent="0.2">
@@ -15099,19 +15105,19 @@
     </row>
     <row r="166" spans="1:30" x14ac:dyDescent="0.2">
       <c r="B166" s="38" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C166" s="31" t="s">
         <v>162</v>
       </c>
       <c r="AA166" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="AB166" s="42" t="s">
+        <v>350</v>
+      </c>
+      <c r="AC166" s="43" t="s">
         <v>351</v>
-      </c>
-      <c r="AB166" s="42" t="s">
-        <v>352</v>
-      </c>
-      <c r="AC166" s="43" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="167" spans="1:30" x14ac:dyDescent="0.2">
@@ -15166,6 +15172,28 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E77:E79"/>
+    <mergeCell ref="Y5:Z5"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="V5:W5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="AE4:AG4"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="C45:C48"/>
+    <mergeCell ref="C69:C72"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="C75:C78"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="C63:C66"/>
     <mergeCell ref="B108:B111"/>
     <mergeCell ref="C108:C111"/>
     <mergeCell ref="B56:B59"/>
@@ -15177,28 +15205,6 @@
     <mergeCell ref="C103:C106"/>
     <mergeCell ref="B97:B100"/>
     <mergeCell ref="C97:C100"/>
-    <mergeCell ref="C45:C48"/>
-    <mergeCell ref="C69:C72"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="C75:C78"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="B69:B72"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="C63:C66"/>
-    <mergeCell ref="AE4:AG4"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="Y5:Z5"/>
-    <mergeCell ref="P5:Q5"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="V5:W5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E30:E31"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
minor changes to BCL variable names
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23EC696A-A193-624B-9453-D312CE5757B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F567B6-661C-3247-9ABD-06B026644296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-960" yWindow="760" windowWidth="34480" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="2340" yWindow="500" windowWidth="34480" windowHeight="19440" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="521">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -1393,9 +1393,6 @@
     <t>\gamma(v)</t>
   </si>
   <si>
-    <t>Vector (dim $2$) storing available stock factor per unit area in healthy forest. Used to determine when average stocks fall below thresholds.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vector (dim $2$) storing initial steady-state storage in each class. Used in integration targets for NPP curve and as initial carbon storage condition. </t>
   </si>
   <si>
@@ -1601,6 +1598,12 @@
   </si>
   <si>
     <t>Vector ($n_T$)  storing removal behavioral adjustment factor (RBAF). Unmet demand from removals could lead to reductions in demand going forward as consumers switch to different fuels. The behavioral adjustment factor allows this behavior to be reflected in changes to demands. A value of $\beta = 1$ means that shifts incurred in the previous time period are totally adopted, while a value of $\beta = 0$ means that exogenous demands remain.</t>
+  </si>
+  <si>
+    <t>x1</t>
+  </si>
+  <si>
+    <t>Vector (dim $2$) storing available stock factor per unit area in healthy forest, or carbon carrying capacity stock factor. Used to determine when average stocks fall below thresholds.</t>
   </si>
 </sst>
 </file>
@@ -7845,7 +7848,7 @@
         <v>405</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C12" s="28"/>
       <c r="G12" s="4">
@@ -7905,10 +7908,10 @@
         <v>116</v>
       </c>
       <c r="AA12" s="38" t="s">
+        <v>452</v>
+      </c>
+      <c r="AB12" s="42" t="s">
         <v>453</v>
-      </c>
-      <c r="AB12" s="42" t="s">
-        <v>454</v>
       </c>
       <c r="AC12" s="43"/>
       <c r="AE12" s="19"/>
@@ -8040,7 +8043,7 @@
       </c>
       <c r="AA14" s="38"/>
       <c r="AB14" s="51" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AC14" s="43" t="s">
         <v>328</v>
@@ -8394,7 +8397,7 @@
         <v>432</v>
       </c>
       <c r="AB21" s="42" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="AC21" s="43" t="s">
         <v>332</v>
@@ -8433,7 +8436,7 @@
         <v>449</v>
       </c>
       <c r="AB22" s="42" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AC22" s="44" t="s">
         <v>342</v>
@@ -8505,10 +8508,10 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA24" s="38" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="AB24" s="42" t="s">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AC24" s="43" t="s">
         <v>331</v>
@@ -8831,7 +8834,7 @@
         <v>405</v>
       </c>
       <c r="B31" s="38" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C31" s="31" t="s">
         <v>162</v>
@@ -8856,7 +8859,7 @@
         <v>413</v>
       </c>
       <c r="AB31" s="42" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AC31" s="43" t="s">
         <v>343</v>
@@ -8867,7 +8870,7 @@
         <v>405</v>
       </c>
       <c r="B32" s="38" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C32" s="31" t="s">
         <v>162</v>
@@ -8878,10 +8881,10 @@
         <v>0.61538461538461542</v>
       </c>
       <c r="AA32" s="38" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AB32" s="42" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="AC32" s="43" t="s">
         <v>343</v>
@@ -8892,20 +8895,20 @@
         <v>405</v>
       </c>
       <c r="B33" s="38" t="s">
+        <v>489</v>
+      </c>
+      <c r="C33" s="31" t="s">
         <v>490</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>491</v>
       </c>
       <c r="E33" s="26"/>
       <c r="G33" s="4">
         <v>0.5</v>
       </c>
       <c r="AA33" s="38" t="s">
+        <v>491</v>
+      </c>
+      <c r="AB33" s="42" t="s">
         <v>492</v>
-      </c>
-      <c r="AB33" s="42" t="s">
-        <v>493</v>
       </c>
       <c r="AC33" s="43" t="s">
         <v>339</v>
@@ -8970,7 +8973,7 @@
         <v>279</v>
       </c>
       <c r="AB35" s="42" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="AC35" s="43" t="s">
         <v>333</v>
@@ -8981,7 +8984,7 @@
         <v>405</v>
       </c>
       <c r="B36" s="38" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C36" s="33" t="s">
         <v>163</v>
@@ -9017,10 +9020,10 @@
         <v>224809.55611554152</v>
       </c>
       <c r="AA36" s="38" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AB36" s="42" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="AC36" s="43" t="s">
         <v>333</v>
@@ -9031,10 +9034,10 @@
         <v>405</v>
       </c>
       <c r="B37" s="38" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="G37" s="4">
         <v>0.14000000000000001</v>
@@ -9058,13 +9061,13 @@
         <v>0.14199999999999999</v>
       </c>
       <c r="AA37" s="38" t="s">
+        <v>511</v>
+      </c>
+      <c r="AB37" s="42" t="s">
+        <v>509</v>
+      </c>
+      <c r="AC37" s="43" t="s">
         <v>512</v>
-      </c>
-      <c r="AB37" s="42" t="s">
-        <v>510</v>
-      </c>
-      <c r="AC37" s="43" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="38" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -9072,10 +9075,10 @@
         <v>405</v>
       </c>
       <c r="B38" s="38" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="G38" s="4">
         <v>1</v>
@@ -9099,13 +9102,13 @@
         <v>1</v>
       </c>
       <c r="AA38" s="38" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="AB38" s="42" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="AC38" s="43" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="39" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -9113,7 +9116,7 @@
         <v>405</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C39" s="31" t="s">
         <v>162</v>
@@ -9141,13 +9144,13 @@
         <v>0.5</v>
       </c>
       <c r="AA39" s="38" t="s">
+        <v>466</v>
+      </c>
+      <c r="AB39" s="42" t="s">
         <v>467</v>
       </c>
-      <c r="AB39" s="42" t="s">
-        <v>468</v>
-      </c>
       <c r="AC39" s="43" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="40" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -9159,7 +9162,7 @@
         <v>405</v>
       </c>
       <c r="B41" s="38" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C41" s="28" t="s">
         <v>174</v>
@@ -9195,13 +9198,13 @@
         <v>8.9210141315691077E-2</v>
       </c>
       <c r="AA41" s="38" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="AB41" s="42" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AC41" s="43" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -11607,7 +11610,7 @@
         <v>405</v>
       </c>
       <c r="B97" s="52" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C97" s="53" t="s">
         <v>174</v>
@@ -11647,7 +11650,7 @@
         <v>437</v>
       </c>
       <c r="AB97" s="42" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AC97" s="43" t="s">
         <v>304</v>
@@ -11772,7 +11775,7 @@
         <v>405</v>
       </c>
       <c r="B101" s="37" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C101" s="28"/>
       <c r="F101" s="14"/>
@@ -11808,7 +11811,7 @@
         <v>436</v>
       </c>
       <c r="AB101" s="42" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="AC101" s="43" t="s">
         <v>435</v>
@@ -13110,7 +13113,7 @@
         <v>7242.7880378741747</v>
       </c>
       <c r="AA128" s="38" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="AB128" s="42" t="s">
         <v>363</v>
@@ -13189,10 +13192,10 @@
         <v>1044</v>
       </c>
       <c r="AA129" s="38" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AB129" s="42" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="AC129" s="43" t="s">
         <v>308</v>
@@ -13268,10 +13271,10 @@
         <v>4339.1516265119217</v>
       </c>
       <c r="AA130" s="38" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="AB130" s="42" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="AC130" s="43" t="s">
         <v>308</v>
@@ -13279,10 +13282,10 @@
     </row>
     <row r="131" spans="1:29" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="50" t="s">
-        <v>405</v>
+        <v>519</v>
       </c>
       <c r="B131" s="38" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C131" s="33" t="s">
         <v>163</v>
@@ -13398,7 +13401,7 @@
         <v>0.4481607219000015</v>
       </c>
       <c r="AA132" s="38" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AB132" s="42" t="s">
         <v>364</v>
@@ -13477,7 +13480,7 @@
         <v>4921079.9272040259</v>
       </c>
       <c r="AA133" s="38" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="AB133" s="42" t="s">
         <v>318</v>
@@ -13516,7 +13519,7 @@
         <v>405</v>
       </c>
       <c r="B136" s="38" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C136" s="28" t="s">
         <v>174</v>
@@ -13551,10 +13554,10 @@
         <v>215127.42331256883</v>
       </c>
       <c r="AA136" s="38" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="AB136" s="42" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="AC136" s="43" t="s">
         <v>333</v>
@@ -13565,7 +13568,7 @@
         <v>405</v>
       </c>
       <c r="B137" s="38" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C137" s="28" t="s">
         <v>174</v>
@@ -13600,10 +13603,10 @@
         <v>9423.9320294407444</v>
       </c>
       <c r="AA137" s="38" t="s">
+        <v>497</v>
+      </c>
+      <c r="AB137" s="42" t="s">
         <v>498</v>
-      </c>
-      <c r="AB137" s="42" t="s">
-        <v>499</v>
       </c>
       <c r="AC137" s="43" t="s">
         <v>315</v>
@@ -13614,7 +13617,7 @@
         <v>405</v>
       </c>
       <c r="B138" s="38" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C138" s="28" t="s">
         <v>174</v>
@@ -13665,7 +13668,7 @@
         <v>405</v>
       </c>
       <c r="B139" s="38" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C139" s="28" t="s">
         <v>174</v>
@@ -13700,10 +13703,10 @@
         <v>0</v>
       </c>
       <c r="AA139" s="38" t="s">
+        <v>473</v>
+      </c>
+      <c r="AB139" s="42" t="s">
         <v>474</v>
-      </c>
-      <c r="AB139" s="42" t="s">
-        <v>475</v>
       </c>
       <c r="AC139" s="43" t="s">
         <v>315</v>
@@ -13751,7 +13754,7 @@
         <v>192920.79914218979</v>
       </c>
       <c r="AA140" s="38" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="AB140" s="42" t="s">
         <v>395</v>
@@ -13816,7 +13819,7 @@
         <v>405</v>
       </c>
       <c r="B142" s="38" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C142" s="28" t="s">
         <v>174</v>
@@ -13853,10 +13856,10 @@
         <v>0</v>
       </c>
       <c r="AA142" s="38" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="AB142" s="42" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="AC142" s="43" t="s">
         <v>315</v>
@@ -14284,7 +14287,7 @@
         <v>186224.98890231474</v>
       </c>
       <c r="AA149" s="38" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AB149" s="42" t="s">
         <v>368</v>
@@ -14366,13 +14369,13 @@
         <v>192920.79914218979</v>
       </c>
       <c r="AA150" s="38" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="AB150" s="42" t="s">
         <v>320</v>
       </c>
       <c r="AC150" s="43" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="151" spans="1:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14484,7 +14487,7 @@
         <v>405</v>
       </c>
       <c r="B154" s="38" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C154" s="33" t="s">
         <v>163</v>
@@ -14552,7 +14555,7 @@
         <v>433</v>
       </c>
       <c r="AB154" s="42" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AC154" s="43" t="s">
         <v>304</v>
@@ -14563,7 +14566,7 @@
         <v>405</v>
       </c>
       <c r="B155" s="38" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C155" s="33" t="s">
         <v>163</v>
@@ -14628,7 +14631,7 @@
         <v>434</v>
       </c>
       <c r="AB155" s="42" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="AC155" s="43" t="s">
         <v>304</v>
@@ -15061,7 +15064,7 @@
         <v>212026.86397460321</v>
       </c>
       <c r="AA164" s="38" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="AB164" s="42" t="s">
         <v>397</v>

</xml_diff>